<commit_message>
[add] 添加 XlsxExcelReaderTest.cs 文件 [mod] 修改 TestXlsxFileReaderFixture.cs 文件
</commit_message>
<xml_diff>
--- a/NPOI API Package Test/NPOIExcelTestProject/TestExcelFiles/TestXlsxFile.xlsx
+++ b/NPOI API Package Test/NPOIExcelTestProject/TestExcelFiles/TestXlsxFile.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\测试\npoi-api-package-test\NPOI API Package Test\NPOIExcelTestProject\TestExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\文档\程序\C#\npoi-api-package-test\NPOI API Package Test\NPOIExcelTestProject\TestExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2444A2E9-8AE5-469A-A159-65CE2DA64220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36DB170-4553-439F-8DEB-58229585D732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A93978CB-B2FB-4F59-901D-F43C525DB99B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{A93978CB-B2FB-4F59-901D-F43C525DB99B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -94,40 +95,40 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="33">
     <numFmt numFmtId="176" formatCode="[$-409]h:mm\ AM/PM;@"/>
-    <numFmt numFmtId="179" formatCode="h&quot;时&quot;mm&quot;分&quot;ss&quot;秒&quot;;@"/>
-    <numFmt numFmtId="181" formatCode="[$-804]aaaa;@"/>
-    <numFmt numFmtId="182" formatCode="[$-409]mmmmm\-yy;@"/>
-    <numFmt numFmtId="183" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="184" formatCode="[DBNum1][$-804]yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
-    <numFmt numFmtId="185" formatCode="[$-409]mmmm\-yy;@"/>
-    <numFmt numFmtId="186" formatCode="[$-409]mmmmm;@"/>
-    <numFmt numFmtId="188" formatCode="[DBNum1][$-804]yyyy&quot;年&quot;m&quot;月&quot;;@"/>
-    <numFmt numFmtId="189" formatCode="[DBNum1][$-804]m&quot;月&quot;d&quot;日&quot;;@"/>
-    <numFmt numFmtId="190" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
-    <numFmt numFmtId="191" formatCode="yyyy&quot;年&quot;m&quot;月&quot;;@"/>
-    <numFmt numFmtId="192" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
-    <numFmt numFmtId="193" formatCode="[$-804]aaa;@"/>
-    <numFmt numFmtId="194" formatCode="yyyy/m/d;@"/>
-    <numFmt numFmtId="195" formatCode="[$-409]yyyy/m/d\ h:mm\ AM/PM;@"/>
-    <numFmt numFmtId="196" formatCode="yyyy/m/d\ h:mm;@"/>
-    <numFmt numFmtId="197" formatCode="yy/m/d;@"/>
-    <numFmt numFmtId="198" formatCode="m/d;@"/>
-    <numFmt numFmtId="199" formatCode="m/d/yy;@"/>
-    <numFmt numFmtId="200" formatCode="mm/dd/yy;@"/>
-    <numFmt numFmtId="201" formatCode="[$-409]d\-mmm;@"/>
-    <numFmt numFmtId="202" formatCode="[$-409]d\-mmm\-yy;@"/>
-    <numFmt numFmtId="203" formatCode="[$-409]dd\-mmm\-yy;@"/>
-    <numFmt numFmtId="204" formatCode="[$-409]mmm\-yy;@"/>
-    <numFmt numFmtId="205" formatCode="h:mm;@"/>
-    <numFmt numFmtId="206" formatCode="h:mm:ss;@"/>
-    <numFmt numFmtId="207" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="208" formatCode="h&quot;时&quot;mm&quot;分&quot;;@"/>
-    <numFmt numFmtId="209" formatCode="上午/下午h&quot;时&quot;mm&quot;分&quot;;@"/>
-    <numFmt numFmtId="210" formatCode="上午/下午h&quot;时&quot;mm&quot;分&quot;ss&quot;秒&quot;;@"/>
-    <numFmt numFmtId="211" formatCode="[DBNum1][$-804]h&quot;时&quot;mm&quot;分&quot;;@"/>
-    <numFmt numFmtId="212" formatCode="[DBNum1][$-804]上午/下午h&quot;时&quot;mm&quot;分&quot;;@"/>
+    <numFmt numFmtId="177" formatCode="h&quot;时&quot;mm&quot;分&quot;ss&quot;秒&quot;;@"/>
+    <numFmt numFmtId="178" formatCode="[$-804]aaaa;@"/>
+    <numFmt numFmtId="179" formatCode="[$-409]mmmmm\-yy;@"/>
+    <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="181" formatCode="[DBNum1][$-804]yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="182" formatCode="[$-409]mmmm\-yy;@"/>
+    <numFmt numFmtId="183" formatCode="[$-409]mmmmm;@"/>
+    <numFmt numFmtId="184" formatCode="[DBNum1][$-804]yyyy&quot;年&quot;m&quot;月&quot;;@"/>
+    <numFmt numFmtId="185" formatCode="[DBNum1][$-804]m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="186" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="187" formatCode="yyyy&quot;年&quot;m&quot;月&quot;;@"/>
+    <numFmt numFmtId="188" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="189" formatCode="[$-804]aaa;@"/>
+    <numFmt numFmtId="190" formatCode="yyyy/m/d;@"/>
+    <numFmt numFmtId="191" formatCode="[$-409]yyyy/m/d\ h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="192" formatCode="yyyy/m/d\ h:mm;@"/>
+    <numFmt numFmtId="193" formatCode="yy/m/d;@"/>
+    <numFmt numFmtId="194" formatCode="m/d;@"/>
+    <numFmt numFmtId="195" formatCode="m/d/yy;@"/>
+    <numFmt numFmtId="196" formatCode="mm/dd/yy;@"/>
+    <numFmt numFmtId="197" formatCode="[$-409]d\-mmm;@"/>
+    <numFmt numFmtId="198" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="199" formatCode="[$-409]dd\-mmm\-yy;@"/>
+    <numFmt numFmtId="200" formatCode="[$-409]mmm\-yy;@"/>
+    <numFmt numFmtId="201" formatCode="h:mm;@"/>
+    <numFmt numFmtId="202" formatCode="h:mm:ss;@"/>
+    <numFmt numFmtId="203" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="204" formatCode="h&quot;时&quot;mm&quot;分&quot;;@"/>
+    <numFmt numFmtId="205" formatCode="上午/下午h&quot;时&quot;mm&quot;分&quot;;@"/>
+    <numFmt numFmtId="206" formatCode="上午/下午h&quot;时&quot;mm&quot;分&quot;ss&quot;秒&quot;;@"/>
+    <numFmt numFmtId="207" formatCode="[DBNum1][$-804]h&quot;时&quot;mm&quot;分&quot;;@"/>
+    <numFmt numFmtId="208" formatCode="[DBNum1][$-804]上午/下午h&quot;时&quot;mm&quot;分&quot;;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +145,12 @@
       <sz val="9"/>
       <name val="等线"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -166,95 +173,101 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="189" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="190" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="191" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="192" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="193" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="194" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="196" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="197" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="198" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="199" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="190" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="191" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="192" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="193" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="194" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="196" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="197" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="198" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="199" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -264,31 +277,10 @@
     <xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="210" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="211" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -567,36 +559,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4540F915-C332-45C4-AC0D-4AF5870E8D87}">
   <dimension ref="A1:X6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.58203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.75" style="1" customWidth="1"/>
     <col min="4" max="4" width="15" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.75" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.4140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.08203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.9140625" style="1" customWidth="1"/>
     <col min="10" max="10" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="19.77734375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.75" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19.75" style="1" customWidth="1"/>
     <col min="13" max="13" width="15" style="1" customWidth="1"/>
-    <col min="14" max="14" width="9.44140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="5.109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="9.4140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.08203125" style="1" customWidth="1"/>
     <col min="16" max="16" width="7.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="8.6640625" style="1" customWidth="1"/>
     <col min="18" max="18" width="9" style="1" customWidth="1"/>
     <col min="19" max="19" width="11" style="1" customWidth="1"/>
     <col min="20" max="20" width="10.6640625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="8.21875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="6.109375" style="1" customWidth="1"/>
+    <col min="21" max="21" width="8.25" style="1" customWidth="1"/>
+    <col min="22" max="22" width="11.4140625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="6.08203125" style="1" customWidth="1"/>
     <col min="24" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="b">
@@ -606,8 +598,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1">
@@ -617,128 +609,127 @@
         <v>123.456</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
-        <v>45658.5</v>
-      </c>
-      <c r="C3" s="5">
-        <v>45658.5</v>
-      </c>
-      <c r="D3" s="6">
-        <v>45658.5</v>
-      </c>
-      <c r="E3" s="7">
-        <v>45658.5</v>
-      </c>
-      <c r="F3" s="8">
-        <v>45658.5</v>
-      </c>
-      <c r="G3" s="9">
-        <v>45658.5</v>
-      </c>
-      <c r="H3" s="10">
-        <v>45658.5</v>
-      </c>
-      <c r="I3" s="11">
-        <v>45658.5</v>
-      </c>
-      <c r="J3" s="12">
-        <v>45658.5</v>
-      </c>
-      <c r="K3" s="13">
-        <v>45658.5</v>
-      </c>
-      <c r="L3" s="14">
-        <v>45658.5</v>
-      </c>
-      <c r="M3" s="15">
-        <v>45658.5</v>
-      </c>
-      <c r="N3" s="16">
-        <v>45658.5</v>
-      </c>
-      <c r="O3" s="17">
-        <v>45658.5</v>
-      </c>
-      <c r="P3" s="18">
-        <v>45658.5</v>
-      </c>
-      <c r="Q3" s="19">
-        <v>45658.5</v>
-      </c>
-      <c r="R3" s="20">
-        <v>45658.5</v>
-      </c>
-      <c r="S3" s="21">
-        <v>45658.5</v>
-      </c>
-      <c r="T3" s="22">
-        <v>45658.5</v>
-      </c>
-      <c r="U3" s="24">
-        <v>45658.5</v>
-      </c>
-      <c r="V3" s="25">
-        <v>45658.5</v>
-      </c>
-      <c r="W3" s="26">
-        <v>45658.5</v>
-      </c>
-      <c r="X3" s="27">
+      <c r="B3" s="2">
+        <v>45658.5</v>
+      </c>
+      <c r="C3" s="3">
+        <v>45658.5</v>
+      </c>
+      <c r="D3" s="4">
+        <v>45658.5</v>
+      </c>
+      <c r="E3" s="5">
+        <v>45658.5</v>
+      </c>
+      <c r="F3" s="6">
+        <v>45658.5</v>
+      </c>
+      <c r="G3" s="7">
+        <v>45658.5</v>
+      </c>
+      <c r="H3" s="8">
+        <v>45658.5</v>
+      </c>
+      <c r="I3" s="9">
+        <v>45658.5</v>
+      </c>
+      <c r="J3" s="10">
+        <v>45658.5</v>
+      </c>
+      <c r="K3" s="11">
+        <v>45658.5</v>
+      </c>
+      <c r="L3" s="12">
+        <v>45658.5</v>
+      </c>
+      <c r="M3" s="13">
+        <v>45658.5</v>
+      </c>
+      <c r="N3" s="14">
+        <v>45658.5</v>
+      </c>
+      <c r="O3" s="15">
+        <v>45658.5</v>
+      </c>
+      <c r="P3" s="16">
+        <v>45658.5</v>
+      </c>
+      <c r="Q3" s="17">
+        <v>45658.5</v>
+      </c>
+      <c r="R3" s="18">
+        <v>45658.5</v>
+      </c>
+      <c r="S3" s="19">
+        <v>45658.5</v>
+      </c>
+      <c r="T3" s="20">
+        <v>45658.5</v>
+      </c>
+      <c r="U3" s="21">
+        <v>45658.5</v>
+      </c>
+      <c r="V3" s="22">
+        <v>45658.5</v>
+      </c>
+      <c r="W3" s="23">
+        <v>45658.5</v>
+      </c>
+      <c r="X3" s="24">
         <v>45659</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="28">
-        <v>45658.5</v>
-      </c>
-      <c r="C4" s="29">
-        <v>45658.5</v>
-      </c>
-      <c r="D4" s="30">
-        <v>45658.5</v>
-      </c>
-      <c r="E4" s="31">
-        <v>45658.5</v>
-      </c>
-      <c r="F4" s="32">
-        <v>45658.5</v>
-      </c>
-      <c r="G4" s="33">
-        <v>45658.5</v>
-      </c>
-      <c r="H4" s="34">
-        <v>45658.5</v>
-      </c>
-      <c r="I4" s="35">
-        <v>45658.5</v>
-      </c>
-      <c r="J4" s="36">
-        <v>45658.5</v>
-      </c>
-      <c r="K4" s="37">
-        <v>45658.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
+      <c r="B4" s="25">
+        <v>45658.5</v>
+      </c>
+      <c r="C4" s="26">
+        <v>45658.5</v>
+      </c>
+      <c r="D4" s="27">
+        <v>45658.5</v>
+      </c>
+      <c r="E4" s="28">
+        <v>45658.5</v>
+      </c>
+      <c r="F4" s="29">
+        <v>45658.5</v>
+      </c>
+      <c r="G4" s="30">
+        <v>45658.5</v>
+      </c>
+      <c r="H4" s="31">
+        <v>45658.5</v>
+      </c>
+      <c r="I4" s="32">
+        <v>45658.5</v>
+      </c>
+      <c r="J4" s="33">
+        <v>45658.5</v>
+      </c>
+      <c r="K4" s="34">
+        <v>45658.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" s="38" t="s">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="38"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -750,17 +741,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2596702-03B5-4022-90E8-827EB28B99A3}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="1" customWidth="1"/>
-    <col min="2" max="4" width="17.44140625" style="1" customWidth="1"/>
+    <col min="2" max="4" width="17.4140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="1" t="b">
@@ -772,9 +763,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="41"/>
-      <c r="B2" s="39" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="36"/>
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="1">
@@ -782,19 +773,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="41"/>
-      <c r="B3" s="39" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="36"/>
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="40">
+      <c r="C3" s="35">
         <f>DATE(2025,1,1) + TIME(12,0,0)</f>
         <v>45658.5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="41"/>
-      <c r="B4" s="39" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="36"/>
+      <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="1" t="e">
@@ -802,9 +793,9 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="41"/>
-      <c r="B5" s="39" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="36"/>
+      <c r="B5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="1" t="str">
@@ -823,4 +814,14 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A4DAFE7-2627-4872-847D-B8F5C7A19B1D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[mod] 添加 SheetReader.cs 的单元测试
</commit_message>
<xml_diff>
--- a/NPOI API Package Test/NPOIExcelTestProject/TestExcelFiles/TestXlsxFile.xlsx
+++ b/NPOI API Package Test/NPOIExcelTestProject/TestExcelFiles/TestXlsxFile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\测试\npoi-api-package-test\NPOI API Package Test\NPOIExcelTestProject\TestExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4D77C3-F5F5-4F80-ACF0-ADFECA61A0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED6A5EEC-7335-40A0-B3B0-5373EC9ABCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A93978CB-B2FB-4F59-901D-F43C525DB99B}"/>
   </bookViews>
@@ -89,18 +89,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>编号</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>姓名</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>年纪</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>张三</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -122,6 +110,18 @@
   </si>
   <si>
     <t>刘八</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Age</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -899,13 +899,13 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="37" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D2" s="37" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -914,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3" s="36">
         <v>20</v>
@@ -925,7 +925,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D4" s="36">
         <v>21</v>
@@ -936,7 +936,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D5" s="36">
         <v>25</v>
@@ -947,7 +947,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D6" s="36">
         <v>19</v>
@@ -958,7 +958,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D7" s="36">
         <v>23</v>
@@ -969,7 +969,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D8" s="36">
         <v>24</v>

</xml_diff>